<commit_message>
Misc updates — BrandGrid, PurchaseModal, inquiries, config
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/products-template.xlsx
+++ b/backend/products-template.xlsx
@@ -398,32 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W3"/>
-  <cols>
-    <col min="1" max="1" width="18.83203125" customWidth="1"/>
-    <col min="2" max="2" width="18.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="18.83203125" customWidth="1"/>
-    <col min="5" max="5" width="18.83203125" customWidth="1"/>
-    <col min="6" max="6" width="18.83203125" customWidth="1"/>
-    <col min="7" max="7" width="18.83203125" customWidth="1"/>
-    <col min="8" max="8" width="18.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" customWidth="1"/>
-    <col min="11" max="11" width="18.83203125" customWidth="1"/>
-    <col min="12" max="12" width="18.83203125" customWidth="1"/>
-    <col min="13" max="13" width="18.83203125" customWidth="1"/>
-    <col min="14" max="14" width="18.83203125" customWidth="1"/>
-    <col min="15" max="15" width="18.83203125" customWidth="1"/>
-    <col min="16" max="16" width="18.83203125" customWidth="1"/>
-    <col min="17" max="17" width="18.83203125" customWidth="1"/>
-    <col min="18" max="18" width="18.83203125" customWidth="1"/>
-    <col min="19" max="19" width="18.83203125" customWidth="1"/>
-    <col min="20" max="20" width="18.83203125" customWidth="1"/>
-    <col min="21" max="21" width="18.83203125" customWidth="1"/>
-    <col min="22" max="22" width="18.83203125" customWidth="1"/>
-    <col min="23" max="23" width="18.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:W4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -638,9 +613,80 @@
         <v>B75806</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>crocs-batman-batmobile-classic-clog</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Crocs Batman Batmobile Classic Clog</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Crocs</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Black</v>
+      </c>
+      <c r="E4" t="str">
+        <v>unisex</v>
+      </c>
+      <c r="F4">
+        <v>8299</v>
+      </c>
+      <c r="G4">
+        <v>12000</v>
+      </c>
+      <c r="H4">
+        <v>31</v>
+      </c>
+      <c r="I4" t="str">
+        <v>https://www.crocs.in/media/catalog/product/2/1/210219_001_alt100.jpg?width=820</v>
+      </c>
+      <c r="J4" t="str">
+        <v>https://www.crocs.in/media/catalog/product/2/1/210219_001_alt120_1.jpg?width=820</v>
+      </c>
+      <c r="K4" t="str">
+        <v>4, 5, 6, 7</v>
+      </c>
+      <c r="L4" t="str">
+        <v>4, 5, 6, 7</v>
+      </c>
+      <c r="M4" t="str">
+        <v>black</v>
+      </c>
+      <c r="N4" t="str">
+        <v>crocs,batman,dc,clog,casual</v>
+      </c>
+      <c r="O4" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="P4" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="Q4" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="R4" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="S4">
+        <v>0</v>
+      </c>
+      <c r="T4">
+        <v>0</v>
+      </c>
+      <c r="U4" t="str">
+        <v>The Crocs Batman Batmobile Classic Clog features a bold Batman-inspired design with Batmobile graphics. Built on the iconic Classic Clog silhouette with Croslite foam for lightweight comfort.</v>
+      </c>
+      <c r="V4" t="str">
+        <v>lifestyle</v>
+      </c>
+      <c r="W4" t="str">
+        <v>CROCS-BATMAN-BATMOBILE-210219-001</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W4"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -648,10 +694,6 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B34"/>
-  <cols>
-    <col min="1" max="1" width="30.83203125" customWidth="1"/>
-    <col min="2" max="2" width="80.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">

</xml_diff>

<commit_message>
Add Crocs Batman Batmobile Classic Clog, add Crocs brand support
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/products-template.xlsx
+++ b/backend/products-template.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W4"/>
+  <dimension ref="A1:W2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -473,220 +473,78 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>nike-air-max-90-white-black</v>
+        <v>crocs-batman-batmobile-classic-clog</v>
       </c>
       <c r="B2" t="str">
-        <v>Air Max 90</v>
+        <v>Crocs Batman Batmobile Classic Clog</v>
       </c>
       <c r="C2" t="str">
-        <v>Nike</v>
+        <v>Crocs</v>
       </c>
       <c r="D2" t="str">
-        <v>White / Black / Grey</v>
+        <v>Black</v>
       </c>
       <c r="E2" t="str">
         <v>unisex</v>
       </c>
       <c r="F2">
-        <v>12995</v>
+        <v>8299</v>
       </c>
       <c r="G2">
-        <v>14995</v>
+        <v>12000</v>
       </c>
       <c r="H2">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="I2" t="str">
-        <v>https://images.unsplash.com/photo-1542291026-7eec264c27ff?w=800&amp;q=80, https://images.unsplash.com/photo-1606107557195-0e29a4b5b4aa?w=800&amp;q=80</v>
+        <v>https://djm0962033frr.cloudfront.net/1_51_b5e926126c.webp, https://cdn.shopify.com/s/files/1/0570/7389/3509/t/1/assets/1746890793_1467180_01_jpg.jpeg?v=1746890793, https://cdn.shopify.com/s/files/1/0570/7389/3509/t/1/assets/1746890796_1467180_02_jpg.jpeg?v=1746890797, https://cdn.shopify.com/s/files/1/0570/7389/3509/t/1/assets/1746890800_1467180_03_jpg.jpeg?v=1746890800, https://cdn.shopify.com/s/files/1/0570/7389/3509/t/1/assets/1746890803_1467180_04_jpg.jpeg?v=1746890804, https://cdn.shopify.com/s/files/1/0570/7389/3509/t/1/assets/1746890789_1467180_00_png.png?v=1746890790</v>
       </c>
       <c r="J2" t="str">
-        <v>https://images.unsplash.com/photo-1606107557195-0e29a4b5b4aa?w=800&amp;q=80</v>
+        <v>https://cdn.shopify.com/s/files/1/0570/7389/3509/t/1/assets/1746890796_1467180_02_jpg.jpeg?v=1746890797</v>
       </c>
       <c r="K2" t="str">
-        <v>6, 7, 7.5, 8, 8.5, 9, 9.5, 10, 10.5, 11</v>
+        <v>4, 5, 6, 7</v>
       </c>
       <c r="L2" t="str">
-        <v>7, 8, 8.5, 9, 10</v>
+        <v>4, 5, 6, 7</v>
       </c>
       <c r="M2" t="str">
-        <v>white, black</v>
+        <v>black</v>
       </c>
       <c r="N2" t="str">
-        <v>classic, lifestyle, retro</v>
+        <v>crocs,batman,dc,clog,casual</v>
       </c>
       <c r="O2" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="P2" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="Q2" t="str">
         <v>TRUE</v>
-      </c>
-      <c r="P2" t="str">
-        <v>TRUE</v>
-      </c>
-      <c r="Q2" t="str">
-        <v>FALSE</v>
       </c>
       <c r="R2" t="str">
         <v>FALSE</v>
       </c>
       <c r="S2">
-        <v>4.6</v>
+        <v>0</v>
       </c>
       <c r="T2">
-        <v>312</v>
+        <v>0</v>
       </c>
       <c r="U2" t="str">
-        <v>The Air Max 90 stays true to its OG running roots with the iconic Waffle outsole, stitched overlays, and classic TPU accents.</v>
+        <v>The Crocs Batman Batmobile Classic Clog features a bold Batman-inspired design with Batmobile graphics. Built on the iconic Classic Clog silhouette with Croslite foam for lightweight comfort.</v>
       </c>
       <c r="V2" t="str">
         <v>lifestyle</v>
       </c>
       <c r="W2" t="str">
-        <v>CT4352-100</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>adidas-samba-og-white-black</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Samba OG</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Adidas</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Cloud White / Core Black</v>
-      </c>
-      <c r="E3" t="str">
-        <v>unisex</v>
-      </c>
-      <c r="F3">
-        <v>9995</v>
-      </c>
-      <c r="G3" t="str">
-        <v/>
-      </c>
-      <c r="H3" t="str">
-        <v/>
-      </c>
-      <c r="I3" t="str">
-        <v>https://images.unsplash.com/photo-1539185441755-769473a23570?w=800&amp;q=80</v>
-      </c>
-      <c r="J3" t="str">
-        <v>https://images.unsplash.com/photo-1600269452121-4f2416e55c28?w=800&amp;q=80</v>
-      </c>
-      <c r="K3" t="str">
-        <v>6, 7, 7.5, 8, 8.5, 9, 9.5, 10, 10.5, 11</v>
-      </c>
-      <c r="L3" t="str">
-        <v>7, 8, 9, 10</v>
-      </c>
-      <c r="M3" t="str">
-        <v>white, black</v>
-      </c>
-      <c r="N3" t="str">
-        <v>classic, lifestyle, football</v>
-      </c>
-      <c r="O3" t="str">
-        <v>TRUE</v>
-      </c>
-      <c r="P3" t="str">
-        <v>TRUE</v>
-      </c>
-      <c r="Q3" t="str">
-        <v>FALSE</v>
-      </c>
-      <c r="R3" t="str">
-        <v>FALSE</v>
-      </c>
-      <c r="S3">
-        <v>4.8</v>
-      </c>
-      <c r="T3">
-        <v>1876</v>
-      </c>
-      <c r="U3" t="str">
-        <v>A street icon since 1950. The Adidas Samba OG brings indoor football heritage to everyday style.</v>
-      </c>
-      <c r="V3" t="str">
-        <v>lifestyle</v>
-      </c>
-      <c r="W3" t="str">
-        <v>B75806</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>crocs-batman-batmobile-classic-clog</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Crocs Batman Batmobile Classic Clog</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Crocs</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Black</v>
-      </c>
-      <c r="E4" t="str">
-        <v>unisex</v>
-      </c>
-      <c r="F4">
-        <v>8299</v>
-      </c>
-      <c r="G4">
-        <v>12000</v>
-      </c>
-      <c r="H4">
-        <v>31</v>
-      </c>
-      <c r="I4" t="str">
-        <v>https://www.crocs.in/media/catalog/product/2/1/210219_001_alt100.jpg?width=820</v>
-      </c>
-      <c r="J4" t="str">
-        <v>https://www.crocs.in/media/catalog/product/2/1/210219_001_alt120_1.jpg?width=820</v>
-      </c>
-      <c r="K4" t="str">
-        <v>4, 5, 6, 7</v>
-      </c>
-      <c r="L4" t="str">
-        <v>4, 5, 6, 7</v>
-      </c>
-      <c r="M4" t="str">
-        <v>black</v>
-      </c>
-      <c r="N4" t="str">
-        <v>crocs,batman,dc,clog,casual</v>
-      </c>
-      <c r="O4" t="str">
-        <v>FALSE</v>
-      </c>
-      <c r="P4" t="str">
-        <v>FALSE</v>
-      </c>
-      <c r="Q4" t="str">
-        <v>TRUE</v>
-      </c>
-      <c r="R4" t="str">
-        <v>FALSE</v>
-      </c>
-      <c r="S4">
-        <v>0</v>
-      </c>
-      <c r="T4">
-        <v>0</v>
-      </c>
-      <c r="U4" t="str">
-        <v>The Crocs Batman Batmobile Classic Clog features a bold Batman-inspired design with Batmobile graphics. Built on the iconic Classic Clog silhouette with Croslite foam for lightweight comfort.</v>
-      </c>
-      <c r="V4" t="str">
-        <v>lifestyle</v>
-      </c>
-      <c r="W4" t="str">
         <v>CROCS-BATMAN-BATMOBILE-210219-001</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W2"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>